<commit_message>
Paar sachen in BOM ersetzt
</commit_message>
<xml_diff>
--- a/Dub Siren PCB/Default Configuration/Project Outputs for Dub Siren PCB/BOM/BOM_PartType-Dub Siren PCB.xlsx
+++ b/Dub Siren PCB/Default Configuration/Project Outputs for Dub Siren PCB/BOM/BOM_PartType-Dub Siren PCB.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maxim\Documents\GitHub\Dub-Siren\Dub Siren PCB\Default Configuration\Project Outputs for Dub Siren PCB\BOM\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAB3FA52-FA95-4853-94CE-C053F4B1041D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="45" windowWidth="27795" windowHeight="17175"/>
+    <workbookView xWindow="7140" yWindow="3135" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM_PartType-Dub Siren PCB" sheetId="1" r:id="rId1"/>
@@ -40,27 +46,15 @@
     <t>C5, C8</t>
   </si>
   <si>
-    <t>22p, 0603</t>
-  </si>
-  <si>
     <t>C9, C10, C11, C12, C13, C14, C16, C18</t>
   </si>
   <si>
-    <t>2u2, 0603</t>
-  </si>
-  <si>
     <t>C19, C20</t>
   </si>
   <si>
-    <t>2n2, 0603</t>
-  </si>
-  <si>
     <t>D1, D2</t>
   </si>
   <si>
-    <t>WP424QR51WT/D-AMT</t>
-  </si>
-  <si>
     <t>LED 3mm</t>
   </si>
   <si>
@@ -179,12 +173,25 @@
   </si>
   <si>
     <t>ABM8</t>
+  </si>
+  <si>
+    <t>22pF, 0603</t>
+  </si>
+  <si>
+    <t>2.2uF, 0603</t>
+  </si>
+  <si>
+    <t>2.2nF, 0603</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 	
+XL-302UBD</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -241,16 +248,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -258,14 +268,17 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
   </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -303,7 +316,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -375,7 +388,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -548,9 +561,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D21"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="33.7109375" customWidth="1"/>
     <col min="2" max="2" width="10" customWidth="1"/>
@@ -594,7 +607,7 @@
         <v>2</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>8</v>
+        <v>51</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>6</v>
@@ -602,13 +615,13 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B4" s="3">
         <v>8</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>10</v>
+        <v>52</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>6</v>
@@ -616,240 +629,240 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B5" s="3">
         <v>2</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>12</v>
+        <v>53</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" ht="22.5" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B6" s="3">
         <v>2</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>14</v>
+      <c r="C6" s="4" t="s">
+        <v>54</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="B7" s="3">
         <v>1</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="B8" s="3">
         <v>1</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B9" s="3">
         <v>1</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="B10" s="3">
         <v>1</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B11" s="3">
         <v>5</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="B12" s="3">
         <v>9</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="B13" s="3">
         <v>2</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="B14" s="3">
         <v>10</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="B15" s="3">
         <v>3</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B16" s="3">
         <v>1</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B17" s="3">
         <v>1</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="B18" s="3">
         <v>1</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="B19" s="3">
         <v>1</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="B20" s="3">
         <v>1</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="B21" s="3">
         <v>1</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>

</xml_diff>